<commit_message>
Restyle motor price list Excel to match PDF design
Rework the .xlsx to mirror the source IE4.pdf: IE 4 heading, embedded
AEMOT logo, grey table headers with black borders, rotated Delta 400 /
Y 690 winding-connection text in the left margin, and the red kirmizi
cizgi stepped boundary above the copper-bar/aluminium-injection motors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jc76z8VnHnosKkFctUCrdC
</commit_message>
<xml_diff>
--- a/AEM_Motor_Fiyat_Listesi_09-07-2026.xlsx
+++ b/AEM_Motor_Fiyat_Listesi_09-07-2026.xlsx
@@ -17,9 +17,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;₺&quot;;;&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₺&quot;;;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,47 +29,29 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="11"/>
     </font>
     <font>
-      <color rgb="00FFFFFF"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="12"/>
+      <sz val="30"/>
     </font>
     <font>
       <b val="1"/>
-      <i val="1"/>
-      <color rgb="002E5395"/>
-      <sz val="10"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
     <font>
       <sz val="10"/>
     </font>
-    <font>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -78,31 +60,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E5395"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF0FA"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -112,74 +74,318 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00FF0000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00FF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00FF0000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FF0000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00FF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FF0000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -256,6 +462,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="424331"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -547,1380 +783,1451 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>AEM ELEKTRİK MOTORLARI SAN. VE TİC. A.Ş.</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Taşpınar Kasabası Yavuz Selim Mah. Sümrü Sk. No: 61/1  •  Aksaray / Türkiye  •  Tel: +90 382 288 02 00 (6 hat)  •  Fax: +90 382 266 21 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>3-FAZLI PİK GÖVDELİ ASENKRON ELEKTRİK MOTORLARI — PERAKENDE FİYAT LİSTESİ</t>
+          <t>Taşpınar Kasabası Yavuz Selim Mah.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>IE 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sümrü Sk. No : 61/1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Liste Tarihi: 09.07.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    Aksaray / Türkiye</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Tel  : + 90 382 288 02 00 (6 hat)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>3-FAZLI PİK GÖVDELİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fax : + 90 382 266 21 30</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ASENKRON ELEKTRİK MOTORLARI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>PERAKENDE FİYAT LİSTESİ</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Δ 400 / Y 690</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>GÜÇ</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>2 Kutup — 3000 d/d</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>4 Kutup — 1500 d/d</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>6 Kutup — 1000 d/d</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>2 Kutup - 3000 d/d</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>4 Kutup - 1500 d/d</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>6 Kutup - 1000 d/d</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>kW</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Motor Tipi</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Fiyat (TL)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Motor Tipi</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Fiyat (TL)</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Motor Tipi</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Fiyat (TL)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="11" ht="15.5" customHeight="1">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>3,00</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>4,00</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>ABP 132 S6A</t>
         </is>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="I11" s="15" t="n">
         <v>29991</v>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="12" ht="15.5" customHeight="1">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>4,00</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>5,50</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>ABP 132 M6A</t>
         </is>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="I12" s="15" t="n">
         <v>34083</v>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="13" ht="15.5" customHeight="1">
+      <c r="A13" s="9" t="n"/>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>5,50</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>7,50</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>ABP 132 S2A</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="E13" s="16" t="n">
         <v>33381</v>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>ABP 132 S4A</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="G13" s="16" t="n">
         <v>35395</v>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>ABP 132 M6B</t>
         </is>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="I13" s="15" t="n">
         <v>39060</v>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="14" ht="15.5" customHeight="1">
+      <c r="A14" s="9" t="n"/>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>7,50</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>10,00</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>ABP 132 S2B</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="E14" s="16" t="n">
         <v>37760</v>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>ABP 132 M4A</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="G14" s="16" t="n">
         <v>41600</v>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>ABP 160 M6A</t>
         </is>
       </c>
-      <c r="H11" s="14" t="n">
+      <c r="I14" s="15" t="n">
         <v>57497</v>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="15" ht="15.5" customHeight="1">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>11,00</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>15,00</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>ABP 160 M2A</t>
         </is>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="E15" s="16" t="n">
         <v>54894</v>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>ABP 160 M4A</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="G15" s="16" t="n">
         <v>63957</v>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>ABP 160 L6A</t>
         </is>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="I15" s="15" t="n">
         <v>73346</v>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="16" ht="15.5" customHeight="1">
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>15,00</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>20,00</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>ABP 160 M2B</t>
         </is>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="E16" s="16" t="n">
         <v>62183</v>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>ABP 160 L4A</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="G16" s="16" t="n">
         <v>74958</v>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>ABP 180 L6A</t>
         </is>
       </c>
-      <c r="H13" s="14" t="n">
+      <c r="I16" s="15" t="n">
         <v>80333</v>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="17" ht="15.5" customHeight="1">
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>18,50</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>25,00</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>ABP 160 L2A</t>
         </is>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="E17" s="16" t="n">
         <v>70026</v>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>ABP 180 M4A</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="G17" s="16" t="n">
         <v>85067</v>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>ABP 200 L6A</t>
         </is>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="I17" s="15" t="n">
         <v>105649</v>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+    <row r="18" ht="15.5" customHeight="1">
+      <c r="A18" s="9" t="n"/>
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>22,00</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>30,00</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>ABP 180 M2A</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="E18" s="16" t="n">
         <v>80363</v>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>ABP 180 L4A</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="G18" s="16" t="n">
         <v>87649</v>
       </c>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="H18" s="13" t="inlineStr">
         <is>
           <t>ABP 200 L6B</t>
         </is>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="I18" s="15" t="n">
         <v>114165</v>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="19" ht="15.5" customHeight="1">
+      <c r="A19" s="9" t="n"/>
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>30,00</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>40,00</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>ABP 200 L2A</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="E19" s="16" t="n">
         <v>128724</v>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>ABP 200 L4A</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="G19" s="16" t="n">
         <v>125952</v>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>ABP 225 M6A</t>
         </is>
       </c>
-      <c r="H16" s="10" t="n">
+      <c r="I19" s="15" t="n">
         <v>138172</v>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="20" ht="15.5" customHeight="1">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>37,00</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>50,00</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>ABP 200 L2B</t>
         </is>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="E20" s="16" t="n">
         <v>141236</v>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>ABP 225 S4A</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="G20" s="16" t="n">
         <v>145612</v>
       </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="H20" s="13" t="inlineStr">
         <is>
           <t>ABP 250 M6A</t>
         </is>
       </c>
-      <c r="H17" s="14" t="n">
+      <c r="I20" s="15" t="n">
         <v>178758</v>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="21" ht="15.5" customHeight="1">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>45,00</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>60,00</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>ABP 225 M2A</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="E21" s="16" t="n">
         <v>158044</v>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>ABP 225 M4A</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="G21" s="16" t="n">
         <v>148802</v>
       </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="H21" s="13" t="inlineStr">
         <is>
           <t>ABP 280 S6A</t>
         </is>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="I21" s="15" t="n">
         <v>212077</v>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="22" ht="15.5" customHeight="1">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>55,00</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>75,00</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>ABP 250 M2A</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="E22" s="16" t="n">
         <v>228312</v>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>ABP 250 M4A</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="G22" s="16" t="n">
         <v>228972</v>
       </c>
-      <c r="G19" s="12" t="inlineStr">
+      <c r="H22" s="13" t="inlineStr">
         <is>
           <t>ABP 280 M6A</t>
         </is>
       </c>
-      <c r="H19" s="14" t="n">
+      <c r="I22" s="15" t="n">
         <v>250910</v>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="23" ht="15.5" customHeight="1">
+      <c r="A23" s="9" t="n"/>
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>75,00</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>100,00</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>ABP 280 S2A</t>
         </is>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="E23" s="16" t="n">
         <v>240828</v>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>ABP 280 S4A</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="G23" s="16" t="n">
         <v>243111</v>
       </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr">
         <is>
           <t>ABP 315 S6A</t>
         </is>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="I23" s="15" t="n">
         <v>322455</v>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="24" ht="15.5" customHeight="1">
+      <c r="A24" s="9" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>90,00</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>125,00</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>ABP 280 M2A</t>
         </is>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="E24" s="16" t="n">
         <v>273280</v>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>ABP 280 M4A</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="G24" s="16" t="n">
         <v>265499</v>
       </c>
-      <c r="G21" s="12" t="inlineStr">
+      <c r="H24" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M6A</t>
         </is>
       </c>
-      <c r="H21" s="14" t="n">
+      <c r="I24" s="15" t="n">
         <v>358652</v>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="25" ht="15.5" customHeight="1">
+      <c r="A25" s="9" t="n"/>
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>110,00</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>150,00</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>ABP 315 S2A</t>
         </is>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="E25" s="16" t="n">
         <v>386573</v>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>ABP 315 S4A</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n">
+      <c r="G25" s="16" t="n">
         <v>380072</v>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M6B</t>
         </is>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="I25" s="15" t="n">
         <v>397433</v>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="26" ht="15.5" customHeight="1">
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>132,00</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>175,00</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M2A</t>
         </is>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="E26" s="16" t="n">
         <v>401396</v>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M4A</t>
         </is>
       </c>
-      <c r="F23" s="14" t="n">
+      <c r="G26" s="16" t="n">
         <v>442816</v>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="H26" s="13" t="inlineStr">
         <is>
           <t>ABP 315 L6A</t>
         </is>
       </c>
-      <c r="H23" s="14" t="n">
+      <c r="I26" s="15" t="n">
         <v>452362</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="27" ht="15.5" customHeight="1">
+      <c r="A27" s="9" t="n"/>
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>160,00</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>220,00</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M2B</t>
         </is>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="E27" s="16" t="n">
         <v>422938</v>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>ABP 315 M4B</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="G27" s="17" t="n">
         <v>499622</v>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="H27" s="18" t="inlineStr">
         <is>
           <t>ABP 355 M6A</t>
         </is>
       </c>
-      <c r="H24" s="10" t="n">
+      <c r="I27" s="19" t="n">
         <v>718144</v>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+    <row r="28" ht="15.5" customHeight="1">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>185,00</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>250,00</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>ABP 315 L2A</t>
         </is>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="E28" s="16" t="n">
         <v>462683</v>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>ABP 315 L4A</t>
         </is>
       </c>
-      <c r="F25" s="14" t="n">
+      <c r="G28" s="17" t="n">
         <v>531982</v>
       </c>
-      <c r="G25" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="H28" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I28" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15.5" customHeight="1">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>200,00</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>270,00</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>ABP 315 L2B</t>
         </is>
       </c>
-      <c r="D26" s="10" t="n">
+      <c r="E29" s="16" t="n">
         <v>474668</v>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>ABP 315 L4B</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="G29" s="17" t="n">
         <v>584620</v>
       </c>
-      <c r="G26" s="8" t="inlineStr">
+      <c r="H29" s="20" t="inlineStr">
         <is>
           <t>ABP 355 M6B</t>
         </is>
       </c>
-      <c r="H26" s="10" t="n">
+      <c r="I29" s="15" t="n">
         <v>753259</v>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="30" ht="15.5" customHeight="1">
+      <c r="A30" s="9" t="n"/>
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>250,00</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>340,00</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M2A</t>
         </is>
       </c>
-      <c r="D27" s="14" t="n">
+      <c r="E30" s="16" t="n">
         <v>828151</v>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M4A</t>
         </is>
       </c>
-      <c r="F27" s="14" t="n">
+      <c r="G30" s="17" t="n">
         <v>711315</v>
       </c>
-      <c r="G27" s="12" t="inlineStr">
+      <c r="H30" s="20" t="inlineStr">
         <is>
           <t>ABP 355 M6C</t>
         </is>
       </c>
-      <c r="H27" s="14" t="n">
+      <c r="I30" s="15" t="n">
         <v>875160</v>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="31" ht="15.5" customHeight="1">
+      <c r="A31" s="9" t="n"/>
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>315,00</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>430,00</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M2B</t>
         </is>
       </c>
-      <c r="D28" s="10" t="n">
+      <c r="E31" s="16" t="n">
         <v>898115</v>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="F31" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M4B</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="G31" s="17" t="n">
         <v>839023</v>
       </c>
-      <c r="G28" s="8" t="inlineStr">
+      <c r="H31" s="20" t="inlineStr">
         <is>
           <t>ABP 355 L6A</t>
         </is>
       </c>
-      <c r="H28" s="10" t="n">
+      <c r="I31" s="15" t="n">
         <v>1009652</v>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="32" ht="15.5" customHeight="1">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>355,00</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>483,00</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="D32" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M2C</t>
         </is>
       </c>
-      <c r="D29" s="14" t="n">
+      <c r="E32" s="16" t="n">
         <v>965468</v>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>ABP 355 M4C</t>
         </is>
       </c>
-      <c r="F29" s="14" t="n">
+      <c r="G32" s="17" t="n">
         <v>877861</v>
       </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="H32" s="20" t="inlineStr">
         <is>
           <t>ABP 355 L6B</t>
         </is>
       </c>
-      <c r="H29" s="14" t="n">
+      <c r="I32" s="15" t="n">
         <v>1504394</v>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+    <row r="33" ht="15.5" customHeight="1">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>400,00</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>544,00</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>ABP 355 L2A</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>ABP 355 L4A</t>
         </is>
       </c>
-      <c r="F30" s="10" t="n">
+      <c r="G33" s="17" t="n">
         <v>912043</v>
       </c>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="H33" s="20" t="inlineStr">
         <is>
           <t>ABP 400 L6A</t>
         </is>
       </c>
-      <c r="H30" s="10" t="n">
+      <c r="I33" s="15" t="n">
         <v>1595645</v>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="34" ht="15.5" customHeight="1">
+      <c r="A34" s="9" t="n"/>
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>450,00</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="C34" s="22" t="inlineStr">
         <is>
           <t>612,00</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="D34" s="23" t="inlineStr">
         <is>
           <t>ABP 355 L2B</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
         <is>
           <t>ABP 355 L4B</t>
         </is>
       </c>
-      <c r="F31" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="G34" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15.5" customHeight="1">
+      <c r="A35" s="9" t="n"/>
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>450,00</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>612,00</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L2A</t>
         </is>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="E35" s="16" t="n">
         <v>1668757</v>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L4A</t>
         </is>
       </c>
-      <c r="F32" s="10" t="n">
+      <c r="G35" s="16" t="n">
         <v>1674364</v>
       </c>
-      <c r="G32" s="8" t="inlineStr">
+      <c r="H35" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L6B</t>
         </is>
       </c>
-      <c r="H32" s="10" t="n">
+      <c r="I35" s="15" t="n">
         <v>1834442</v>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="36" ht="15.5" customHeight="1">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>500,00</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>670,00</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L2B</t>
         </is>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="E36" s="16" t="n">
         <v>1768376</v>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L4B</t>
         </is>
       </c>
-      <c r="F33" s="14" t="n">
+      <c r="G36" s="16" t="n">
         <v>1684200</v>
       </c>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="H36" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L6C</t>
         </is>
       </c>
-      <c r="H33" s="14" t="n">
+      <c r="I36" s="15" t="n">
         <v>1902067</v>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
+    <row r="37" ht="15.5" customHeight="1">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>560,00</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>751,00</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L2C</t>
         </is>
       </c>
-      <c r="D34" s="10" t="n">
+      <c r="E37" s="16" t="n">
         <v>1843683</v>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="F37" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L4C</t>
         </is>
       </c>
-      <c r="F34" s="10" t="n">
+      <c r="G37" s="16" t="n">
         <v>1787577</v>
       </c>
-      <c r="G34" s="8" t="inlineStr">
+      <c r="H37" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L6D</t>
         </is>
       </c>
-      <c r="H34" s="10" t="n">
+      <c r="I37" s="15" t="n">
         <v>2152784</v>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="38" ht="15.5" customHeight="1">
+      <c r="A38" s="9" t="n"/>
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>630,00</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>845,00</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L2D</t>
         </is>
       </c>
-      <c r="D35" s="14" t="n">
+      <c r="E38" s="16" t="n">
         <v>2012750</v>
       </c>
-      <c r="E35" s="12" t="inlineStr">
+      <c r="F38" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L4D</t>
         </is>
       </c>
-      <c r="F35" s="14" t="n">
+      <c r="G38" s="16" t="n">
         <v>1888763</v>
       </c>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.5" customHeight="1">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>710,00</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>952,00</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L2E</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
         <is>
           <t>ABP 400 L4E</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.5" customHeight="1">
+      <c r="A40" s="26" t="n"/>
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>750,00</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="C40" s="27" t="inlineStr">
         <is>
           <t>1.005,00</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="D40" s="28" t="inlineStr">
         <is>
           <t>ABP 400 L2F</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
+      <c r="E40" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" s="28" t="inlineStr">
         <is>
           <t>ABP 400 L4F</t>
         </is>
       </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
-        <is>
-          <t>AÇIKLAMALAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="14" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="G40" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" s="30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="13" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
         <is>
           <t>1. Fiyatlarımıza K.D.V. dahil değildir.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="26" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="31" t="inlineStr">
         <is>
           <t>2. Standart dışı imalat taleplerinde liste fiyatları geçerli değildir; özel imalat fiyat farkı listesi geçerlidir.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="16" t="inlineStr">
+    <row r="44" ht="13" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
         <is>
           <t>3. Fiyatlarımız liste tarihi itibari ile geçerlidir bir önceki tarihli listeyi geçersiz kılar.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="16" t="inlineStr">
+    <row r="45" ht="13" customHeight="1">
+      <c r="A45" s="31" t="inlineStr">
         <is>
           <t>4. 200-225-250-280-315-355 Gövde Motorlarda standart termistör (PTC) uygulaması bulunmaktadır.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="31" t="inlineStr">
         <is>
           <t>5. Kırmızı çizginin altında kalan motorlar BAKIR BARALI/Alüminyum enjeksiyon olarak üretimi yapılabilmektedir. Bu motor fiyatları için firmamızla iletişime geçiniz.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>TEKNİK ÖZELLİKLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="14" customHeight="1">
-      <c r="A47" s="17" t="inlineStr">
+    <row r="48" ht="13" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>GERİLİM</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>400 V</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="14" customHeight="1">
-      <c r="A48" s="17" t="inlineStr">
+      <c r="C48" s="32" t="inlineStr">
+        <is>
+          <t>:  400 V</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="13" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>FREKANS</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>50 Hz</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="14" customHeight="1">
-      <c r="A49" s="17" t="inlineStr">
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>:  50 Hz</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="13" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>YAPI BİÇİMİ</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
+      <c r="C50" s="32" t="inlineStr">
+        <is>
+          <t>:  B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="13" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>KORUMA SINIFI</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>IP 55</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="14" customHeight="1">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>:  IP 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="13" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>İZOLASYON SINIFI</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>F (155 °C)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="14" customHeight="1">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="C52" s="32" t="inlineStr">
+        <is>
+          <t>:  F (155 °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="13" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>İŞLETME ŞEKLİ</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>S1</t>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>:  S1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="33">
     <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="D2:F4"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="A46:I46"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C51:H51"/>
-    <mergeCell ref="C52:H52"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="C48:H48"/>
-    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C53:I53"/>
+    <mergeCell ref="A9:A40"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="C49:I49"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="C49:H49"/>
-    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="C51:I51"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="C50:I50"/>
     <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="G7:I7"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Convert motor prices to EUR (list TL x 0.70 / 50)
Apply a 0.70 coefficient and a 50 TL/EUR rate to every list price and
relabel the price columns as Fiyat (EUR); add explanatory note 6. Same
PDF-matching layout, logo, red line and technical sections retained.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jc76z8VnHnosKkFctUCrdC
</commit_message>
<xml_diff>
--- a/AEM_Motor_Fiyat_Listesi_09-07-2026.xlsx
+++ b/AEM_Motor_Fiyat_Listesi_09-07-2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₺&quot;;;&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;;;&quot;-&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -783,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -916,7 +916,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Fiyat (TL)</t>
+          <t>Fiyat (EUR)</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Fiyat (TL)</t>
+          <t>Fiyat (EUR)</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Fiyat (TL)</t>
+          <t>Fiyat (EUR)</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="I11" s="15" t="n">
-        <v>29991</v>
+        <v>419.87</v>
       </c>
     </row>
     <row r="12" ht="15.5" customHeight="1">
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="I12" s="15" t="n">
-        <v>34083</v>
+        <v>477.16</v>
       </c>
     </row>
     <row r="13" ht="15.5" customHeight="1">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E13" s="16" t="n">
-        <v>33381</v>
+        <v>467.33</v>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="G13" s="16" t="n">
-        <v>35395</v>
+        <v>495.53</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="I13" s="15" t="n">
-        <v>39060</v>
+        <v>546.84</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>37760</v>
+        <v>528.64</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="G14" s="16" t="n">
-        <v>41600</v>
+        <v>582.4</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="I14" s="15" t="n">
-        <v>57497</v>
+        <v>804.96</v>
       </c>
     </row>
     <row r="15" ht="15.5" customHeight="1">
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="E15" s="16" t="n">
-        <v>54894</v>
+        <v>768.52</v>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="G15" s="16" t="n">
-        <v>63957</v>
+        <v>895.4</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="I15" s="15" t="n">
-        <v>73346</v>
+        <v>1026.84</v>
       </c>
     </row>
     <row r="16" ht="15.5" customHeight="1">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="E16" s="16" t="n">
-        <v>62183</v>
+        <v>870.5599999999999</v>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="G16" s="16" t="n">
-        <v>74958</v>
+        <v>1049.41</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="I16" s="15" t="n">
-        <v>80333</v>
+        <v>1124.66</v>
       </c>
     </row>
     <row r="17" ht="15.5" customHeight="1">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="E17" s="16" t="n">
-        <v>70026</v>
+        <v>980.36</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="G17" s="16" t="n">
-        <v>85067</v>
+        <v>1190.94</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="I17" s="15" t="n">
-        <v>105649</v>
+        <v>1479.09</v>
       </c>
     </row>
     <row r="18" ht="15.5" customHeight="1">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="E18" s="16" t="n">
-        <v>80363</v>
+        <v>1125.08</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="G18" s="16" t="n">
-        <v>87649</v>
+        <v>1227.09</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="I18" s="15" t="n">
-        <v>114165</v>
+        <v>1598.31</v>
       </c>
     </row>
     <row r="19" ht="15.5" customHeight="1">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="E19" s="16" t="n">
-        <v>128724</v>
+        <v>1802.14</v>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="G19" s="16" t="n">
-        <v>125952</v>
+        <v>1763.33</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="I19" s="15" t="n">
-        <v>138172</v>
+        <v>1934.41</v>
       </c>
     </row>
     <row r="20" ht="15.5" customHeight="1">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="E20" s="16" t="n">
-        <v>141236</v>
+        <v>1977.3</v>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="G20" s="16" t="n">
-        <v>145612</v>
+        <v>2038.57</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="I20" s="15" t="n">
-        <v>178758</v>
+        <v>2502.61</v>
       </c>
     </row>
     <row r="21" ht="15.5" customHeight="1">
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="E21" s="16" t="n">
-        <v>158044</v>
+        <v>2212.62</v>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="G21" s="16" t="n">
-        <v>148802</v>
+        <v>2083.23</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="I21" s="15" t="n">
-        <v>212077</v>
+        <v>2969.08</v>
       </c>
     </row>
     <row r="22" ht="15.5" customHeight="1">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>228312</v>
+        <v>3196.37</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="G22" s="16" t="n">
-        <v>228972</v>
+        <v>3205.61</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="I22" s="15" t="n">
-        <v>250910</v>
+        <v>3512.74</v>
       </c>
     </row>
     <row r="23" ht="15.5" customHeight="1">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="E23" s="16" t="n">
-        <v>240828</v>
+        <v>3371.59</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="G23" s="16" t="n">
-        <v>243111</v>
+        <v>3403.55</v>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="I23" s="15" t="n">
-        <v>322455</v>
+        <v>4514.37</v>
       </c>
     </row>
     <row r="24" ht="15.5" customHeight="1">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="E24" s="16" t="n">
-        <v>273280</v>
+        <v>3825.92</v>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="G24" s="16" t="n">
-        <v>265499</v>
+        <v>3716.99</v>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="I24" s="15" t="n">
-        <v>358652</v>
+        <v>5021.13</v>
       </c>
     </row>
     <row r="25" ht="15.5" customHeight="1">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="E25" s="16" t="n">
-        <v>386573</v>
+        <v>5412.02</v>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="G25" s="16" t="n">
-        <v>380072</v>
+        <v>5321.01</v>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="I25" s="15" t="n">
-        <v>397433</v>
+        <v>5564.06</v>
       </c>
     </row>
     <row r="26" ht="15.5" customHeight="1">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="E26" s="16" t="n">
-        <v>401396</v>
+        <v>5619.54</v>
       </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="G26" s="16" t="n">
-        <v>442816</v>
+        <v>6199.42</v>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="I26" s="15" t="n">
-        <v>452362</v>
+        <v>6333.07</v>
       </c>
     </row>
     <row r="27" ht="15.5" customHeight="1">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="E27" s="16" t="n">
-        <v>422938</v>
+        <v>5921.13</v>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="G27" s="17" t="n">
-        <v>499622</v>
+        <v>6994.71</v>
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="I27" s="19" t="n">
-        <v>718144</v>
+        <v>10054.02</v>
       </c>
     </row>
     <row r="28" ht="15.5" customHeight="1">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="E28" s="16" t="n">
-        <v>462683</v>
+        <v>6477.56</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="G28" s="17" t="n">
-        <v>531982</v>
+        <v>7447.75</v>
       </c>
       <c r="H28" s="20" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="E29" s="16" t="n">
-        <v>474668</v>
+        <v>6645.35</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="G29" s="17" t="n">
-        <v>584620</v>
+        <v>8184.68</v>
       </c>
       <c r="H29" s="20" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="I29" s="15" t="n">
-        <v>753259</v>
+        <v>10545.63</v>
       </c>
     </row>
     <row r="30" ht="15.5" customHeight="1">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="E30" s="16" t="n">
-        <v>828151</v>
+        <v>11594.11</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="G30" s="17" t="n">
-        <v>711315</v>
+        <v>9958.41</v>
       </c>
       <c r="H30" s="20" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="I30" s="15" t="n">
-        <v>875160</v>
+        <v>12252.24</v>
       </c>
     </row>
     <row r="31" ht="15.5" customHeight="1">
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="E31" s="16" t="n">
-        <v>898115</v>
+        <v>12573.61</v>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="G31" s="17" t="n">
-        <v>839023</v>
+        <v>11746.32</v>
       </c>
       <c r="H31" s="20" t="inlineStr">
         <is>
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="I31" s="15" t="n">
-        <v>1009652</v>
+        <v>14135.13</v>
       </c>
     </row>
     <row r="32" ht="15.5" customHeight="1">
@@ -1745,7 +1745,7 @@
         </is>
       </c>
       <c r="E32" s="16" t="n">
-        <v>965468</v>
+        <v>13516.55</v>
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="G32" s="17" t="n">
-        <v>877861</v>
+        <v>12290.05</v>
       </c>
       <c r="H32" s="20" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="I32" s="15" t="n">
-        <v>1504394</v>
+        <v>21061.52</v>
       </c>
     </row>
     <row r="33" ht="15.5" customHeight="1">
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="G33" s="17" t="n">
-        <v>912043</v>
+        <v>12768.6</v>
       </c>
       <c r="H33" s="20" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
         </is>
       </c>
       <c r="I33" s="15" t="n">
-        <v>1595645</v>
+        <v>22339.03</v>
       </c>
     </row>
     <row r="34" ht="15.5" customHeight="1">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="E35" s="16" t="n">
-        <v>1668757</v>
+        <v>23362.6</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="G35" s="16" t="n">
-        <v>1674364</v>
+        <v>23441.1</v>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
         </is>
       </c>
       <c r="I35" s="15" t="n">
-        <v>1834442</v>
+        <v>25682.19</v>
       </c>
     </row>
     <row r="36" ht="15.5" customHeight="1">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="E36" s="16" t="n">
-        <v>1768376</v>
+        <v>24757.26</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -1909,7 +1909,7 @@
         </is>
       </c>
       <c r="G36" s="16" t="n">
-        <v>1684200</v>
+        <v>23578.8</v>
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="I36" s="15" t="n">
-        <v>1902067</v>
+        <v>26628.94</v>
       </c>
     </row>
     <row r="37" ht="15.5" customHeight="1">
@@ -1938,7 +1938,7 @@
         </is>
       </c>
       <c r="E37" s="16" t="n">
-        <v>1843683</v>
+        <v>25811.56</v>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="G37" s="16" t="n">
-        <v>1787577</v>
+        <v>25026.08</v>
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="I37" s="15" t="n">
-        <v>2152784</v>
+        <v>30138.98</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1">
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="E38" s="16" t="n">
-        <v>2012750</v>
+        <v>28178.5</v>
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="G38" s="16" t="n">
-        <v>1888763</v>
+        <v>26442.68</v>
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
@@ -2117,84 +2117,89 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="13" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>GERİLİM</t>
-        </is>
-      </c>
-      <c r="C48" s="32" t="inlineStr">
-        <is>
-          <t>:  400 V</t>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="31" t="inlineStr">
+        <is>
+          <t>6. Fiyatlar 0,70 katsayı uygulanıp 50 TL/EUR kuru ile EUR'ya çevrilmiştir (EUR = Liste TL × 0,70 ÷ 50).</t>
         </is>
       </c>
     </row>
     <row r="49" ht="13" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>FREKANS</t>
+          <t>GERİLİM</t>
         </is>
       </c>
       <c r="C49" s="32" t="inlineStr">
         <is>
-          <t>:  50 Hz</t>
+          <t>:  400 V</t>
         </is>
       </c>
     </row>
     <row r="50" ht="13" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>YAPI BİÇİMİ</t>
+          <t>FREKANS</t>
         </is>
       </c>
       <c r="C50" s="32" t="inlineStr">
         <is>
-          <t>:  B3</t>
+          <t>:  50 Hz</t>
         </is>
       </c>
     </row>
     <row r="51" ht="13" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>KORUMA SINIFI</t>
+          <t>YAPI BİÇİMİ</t>
         </is>
       </c>
       <c r="C51" s="32" t="inlineStr">
         <is>
-          <t>:  IP 55</t>
+          <t>:  B3</t>
         </is>
       </c>
     </row>
     <row r="52" ht="13" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>İZOLASYON SINIFI</t>
+          <t>KORUMA SINIFI</t>
         </is>
       </c>
       <c r="C52" s="32" t="inlineStr">
         <is>
-          <t>:  F (155 °C)</t>
+          <t>:  IP 55</t>
         </is>
       </c>
     </row>
     <row r="53" ht="13" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
+          <t>İZOLASYON SINIFI</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>:  F (155 °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="13" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
           <t>İŞLETME ŞEKLİ</t>
         </is>
       </c>
-      <c r="C53" s="32" t="inlineStr">
+      <c r="C54" s="32" t="inlineStr">
         <is>
           <t>:  S1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A48:B48"/>
+  <mergeCells count="34">
     <mergeCell ref="C52:I52"/>
     <mergeCell ref="D2:F4"/>
-    <mergeCell ref="C48:I48"/>
     <mergeCell ref="A46:I46"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="A51:B51"/>
@@ -2204,8 +2209,10 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="C53:I53"/>
     <mergeCell ref="A9:A40"/>
+    <mergeCell ref="A54:B54"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A47:I47"/>
     <mergeCell ref="C49:I49"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A50:B50"/>
@@ -2213,6 +2220,7 @@
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="C51:I51"/>
     <mergeCell ref="A44:I44"/>
+    <mergeCell ref="C54:I54"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="F9:G9"/>

</xml_diff>